<commit_message>
feat: optimize field report layout and fix evolution chart logic
</commit_message>
<xml_diff>
--- a/Planilhas/Mapeamento Modelos As Built.xlsx
+++ b/Planilhas/Mapeamento Modelos As Built.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFED4D4-8266-42A6-87D5-1DF7D41F93BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{01155B47-A7E1-4A45-B27D-D246D4740F40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{01155B47-A7E1-4A45-B27D-D246D4740F40}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapeamento Modelos As Built" sheetId="1" r:id="rId1"/>
@@ -2114,7 +2114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2196,89 +2196,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="80">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FFC00000"/>
@@ -2323,6 +2245,13 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3184,6 +3113,24 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
@@ -3200,6 +3147,24 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color theme="2" tint="-0.499984740745262"/>
@@ -3212,6 +3177,29 @@
         </top>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0" outline="0">
@@ -3632,23 +3620,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{866C3304-6896-4132-BDE1-D411E5A4A263}" name="Tabela25" displayName="Tabela25" ref="A1:N115" totalsRowShown="0" headerRowDxfId="45" headerRowBorderDxfId="44" tableBorderDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{866C3304-6896-4132-BDE1-D411E5A4A263}" name="Tabela25" displayName="Tabela25" ref="A1:N115" totalsRowShown="0" headerRowDxfId="42" headerRowBorderDxfId="41" tableBorderDxfId="40">
   <autoFilter ref="A1:N115" xr:uid="{89327300-CC3C-407B-B8DD-5A739EFBE9D6}"/>
   <tableColumns count="14">
-    <tableColumn id="15" xr3:uid="{5AB2FB26-0C02-45E3-A502-8A9EEE36A8D5}" name="Número" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{CDD104E0-7374-4B02-A455-C90B238B4B8C}" name="Edificação" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="1" xr3:uid="{301A5D46-16CA-473B-9351-BE1D26A5B07B}" name="Disciplina" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{368F96D9-3561-4C4A-BDAE-3DC551AAFD95}" name="Modelo Base" dataDxfId="36" totalsRowDxfId="35"/>
-    <tableColumn id="13" xr3:uid="{9347F870-C606-474C-8987-C0384A692B8A}" name="IFC" dataDxfId="34" totalsRowDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{CEA48699-571A-47A6-9971-D4417B2AA5F6}" name="Revit" dataDxfId="32" totalsRowDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{655F2B0D-9AF8-46AC-A6AA-1AD4B62F734C}" name="Descrição do Modelo Base" dataDxfId="30" totalsRowDxfId="29"/>
-    <tableColumn id="12" xr3:uid="{62103DAE-1EDF-4611-8E82-DE32DEB36327}" name="Responsável" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{78F12374-C799-4C0D-972B-13CF16F40C2C}" name="Entregas Parciais" dataDxfId="26" totalsRowDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{2EE2DFF0-2B90-4DB7-B752-B26E702853B0}" name="Modelo Final" dataDxfId="24" totalsRowDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{C778F005-66F7-467D-A2DA-7D551EA88DDC}" name="Descrição do Modelo As Built" dataDxfId="22" totalsRowDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{CEE7BB4A-113F-4FCE-A6C3-8383D540FD96}" name="Coluna2" dataDxfId="20" totalsRowDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{7D15D632-8C90-4093-9910-A4D5E8F9B5B7}" name="Coluna3" dataDxfId="18" totalsRowDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{CA1AE1CB-2C05-4D80-930F-CD45B3A2A546}" name="Coluna1" dataDxfId="16" totalsRowDxfId="15"/>
+    <tableColumn id="15" xr3:uid="{5AB2FB26-0C02-45E3-A502-8A9EEE36A8D5}" name="Número" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{CDD104E0-7374-4B02-A455-C90B238B4B8C}" name="Edificação" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{301A5D46-16CA-473B-9351-BE1D26A5B07B}" name="Disciplina" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{368F96D9-3561-4C4A-BDAE-3DC551AAFD95}" name="Modelo Base" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="13" xr3:uid="{9347F870-C606-474C-8987-C0384A692B8A}" name="IFC" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="11" xr3:uid="{CEA48699-571A-47A6-9971-D4417B2AA5F6}" name="Revit" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{655F2B0D-9AF8-46AC-A6AA-1AD4B62F734C}" name="Descrição do Modelo Base" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{62103DAE-1EDF-4611-8E82-DE32DEB36327}" name="Responsável" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{78F12374-C799-4C0D-972B-13CF16F40C2C}" name="Entregas Parciais" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{2EE2DFF0-2B90-4DB7-B752-B26E702853B0}" name="Modelo Final" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{C778F005-66F7-467D-A2DA-7D551EA88DDC}" name="Descrição do Modelo As Built" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{CEE7BB4A-113F-4FCE-A6C3-8383D540FD96}" name="Coluna2" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{7D15D632-8C90-4093-9910-A4D5E8F9B5B7}" name="Coluna3" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{CA1AE1CB-2C05-4D80-930F-CD45B3A2A546}" name="Coluna1" dataDxfId="13" totalsRowDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="Estilo de Tabela 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3669,16 +3657,16 @@
     <tableColumn id="11" xr3:uid="{85490AF5-8126-403B-BE13-89FC51C90B75}" name="Modelo?" dataDxfId="60" totalsRowDxfId="59">
       <calculatedColumnFormula>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{1A6CE1E3-5BB3-44F1-92E4-53348ED08355}" name="Modelo Base" dataDxfId="2" totalsRowDxfId="58">
+    <tableColumn id="4" xr3:uid="{1A6CE1E3-5BB3-44F1-92E4-53348ED08355}" name="Modelo Base" dataDxfId="58" totalsRowDxfId="57">
       <calculatedColumnFormula>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{C8A2D8C7-FE13-455C-8FA0-4376AA7A5157}" name="Modelo Final" dataDxfId="0" totalsRowDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{F30E3CA7-6313-408B-A184-C31D5C85C30D}" name="Observações" dataDxfId="1" totalsRowDxfId="56"/>
-    <tableColumn id="6" xr3:uid="{1FC618B8-85D8-4C25-9D1B-334FDB6DB2FA}" name="Ação" dataDxfId="55" totalsRowDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{0F268795-CE8E-4BAD-AB15-59A607D5B19F}" name="Coluna5" dataDxfId="53" totalsRowDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{0744AAEB-4F03-4CB9-98BF-C41C4C6AEFF9}" name="Coluna2" dataDxfId="51" totalsRowDxfId="50"/>
-    <tableColumn id="9" xr3:uid="{831E94B9-EE21-4189-BE89-3713D15D2568}" name="Coluna3" dataDxfId="49" totalsRowDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{0A0C52AC-AA1C-40A1-90AD-952AFDBBE270}" name="Coluna1" dataDxfId="47" totalsRowDxfId="46"/>
+    <tableColumn id="12" xr3:uid="{C8A2D8C7-FE13-455C-8FA0-4376AA7A5157}" name="Modelo Final" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{F30E3CA7-6313-408B-A184-C31D5C85C30D}" name="Observações" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{1FC618B8-85D8-4C25-9D1B-334FDB6DB2FA}" name="Ação" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{0F268795-CE8E-4BAD-AB15-59A607D5B19F}" name="Coluna5" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="8" xr3:uid="{0744AAEB-4F03-4CB9-98BF-C41C4C6AEFF9}" name="Coluna2" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{831E94B9-EE21-4189-BE89-3713D15D2568}" name="Coluna3" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="10" xr3:uid="{0A0C52AC-AA1C-40A1-90AD-952AFDBBE270}" name="Coluna1" dataDxfId="44" totalsRowDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="Estilo de Tabela 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8026,23 +8014,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H115">
-    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="PENDENTE">
+    <cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="PENDENTE">
       <formula>NOT(ISERROR(SEARCH("PENDENTE",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="LIBERADO">
+    <cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="LIBERADO">
       <formula>NOT(ISERROR(SEARCH("LIBERADO",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16 J45 J62 J79 J91 J104">
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
       <formula>"Não"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
       <formula>"Sim"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2 M2:N2 K3:N115 G63:G64">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18387,7 +18375,7 @@
     </row>
     <row r="240" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A240" s="3">
-        <f t="shared" ref="A240:A303" si="3">A239+1</f>
+        <f t="shared" ref="A240:A288" si="3">A239+1</f>
         <v>239</v>
       </c>
       <c r="B240" s="8">
@@ -18789,15 +18777,15 @@
       <c r="H249" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I249" s="25" t="str">
+      <c r="I249" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J249" s="26" t="str">
+      <c r="J249" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K249" s="26"/>
+      <c r="K249" s="5"/>
       <c r="L249" s="21"/>
       <c r="M249" s="22"/>
       <c r="N249" s="5"/>
@@ -18831,15 +18819,15 @@
       <c r="H250" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I250" s="25" t="str">
+      <c r="I250" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J250" s="26" t="str">
+      <c r="J250" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K250" s="26"/>
+      <c r="K250" s="5"/>
       <c r="L250" s="21"/>
       <c r="M250" s="22"/>
       <c r="N250" s="5"/>
@@ -18873,15 +18861,15 @@
       <c r="H251" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I251" s="25" t="str">
+      <c r="I251" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J251" s="26" t="str">
+      <c r="J251" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K251" s="26"/>
+      <c r="K251" s="5"/>
       <c r="L251" s="21"/>
       <c r="M251" s="22"/>
       <c r="N251" s="5"/>
@@ -18915,15 +18903,15 @@
       <c r="H252" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I252" s="25" t="str">
+      <c r="I252" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J252" s="26" t="str">
+      <c r="J252" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K252" s="26"/>
+      <c r="K252" s="5"/>
       <c r="L252" s="21"/>
       <c r="M252" s="22"/>
       <c r="N252" s="5"/>
@@ -18957,15 +18945,15 @@
       <c r="H253" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I253" s="25" t="str">
+      <c r="I253" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J253" s="26" t="str">
+      <c r="J253" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K253" s="26"/>
+      <c r="K253" s="5"/>
       <c r="L253" s="21"/>
       <c r="M253" s="22"/>
       <c r="N253" s="5"/>
@@ -18999,15 +18987,15 @@
       <c r="H254" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I254" s="25" t="str">
+      <c r="I254" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J254" s="26" t="str">
+      <c r="J254" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K254" s="26"/>
+      <c r="K254" s="5"/>
       <c r="L254" s="21"/>
       <c r="M254" s="22"/>
       <c r="N254" s="5"/>
@@ -19041,15 +19029,15 @@
       <c r="H255" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I255" s="25" t="str">
+      <c r="I255" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J255" s="26" t="str">
+      <c r="J255" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K255" s="26"/>
+      <c r="K255" s="5"/>
       <c r="L255" s="21"/>
       <c r="M255" s="22"/>
       <c r="N255" s="5"/>
@@ -19083,15 +19071,15 @@
       <c r="H256" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I256" s="25" t="str">
+      <c r="I256" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J256" s="26" t="str">
+      <c r="J256" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K256" s="26"/>
+      <c r="K256" s="5"/>
       <c r="L256" s="21"/>
       <c r="M256" s="22"/>
       <c r="N256" s="5"/>
@@ -19125,15 +19113,15 @@
       <c r="H257" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I257" s="25" t="str">
+      <c r="I257" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J257" s="26" t="str">
+      <c r="J257" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K257" s="26"/>
+      <c r="K257" s="5"/>
       <c r="L257" s="21"/>
       <c r="M257" s="22"/>
       <c r="N257" s="5"/>
@@ -19167,15 +19155,15 @@
       <c r="H258" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I258" s="25" t="str">
+      <c r="I258" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J258" s="26" t="str">
+      <c r="J258" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K258" s="26"/>
+      <c r="K258" s="5"/>
       <c r="L258" s="21"/>
       <c r="M258" s="22"/>
       <c r="N258" s="5"/>
@@ -19209,15 +19197,15 @@
       <c r="H259" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I259" s="25" t="str">
+      <c r="I259" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J259" s="26" t="str">
+      <c r="J259" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K259" s="26"/>
+      <c r="K259" s="5"/>
       <c r="L259" s="21"/>
       <c r="M259" s="22"/>
       <c r="N259" s="5"/>
@@ -19251,15 +19239,15 @@
       <c r="H260" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I260" s="25" t="str">
+      <c r="I260" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J260" s="26" t="str">
+      <c r="J260" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K260" s="26"/>
+      <c r="K260" s="5"/>
       <c r="L260" s="21"/>
       <c r="M260" s="22"/>
       <c r="N260" s="5"/>
@@ -19293,15 +19281,15 @@
       <c r="H261" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I261" s="25" t="str">
+      <c r="I261" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J261" s="26" t="str">
+      <c r="J261" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K261" s="26"/>
+      <c r="K261" s="5"/>
       <c r="L261" s="21"/>
       <c r="M261" s="22"/>
       <c r="N261" s="5"/>
@@ -19335,15 +19323,15 @@
       <c r="H262" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I262" s="25" t="str">
+      <c r="I262" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J262" s="26" t="str">
+      <c r="J262" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K262" s="26"/>
+      <c r="K262" s="5"/>
       <c r="L262" s="21"/>
       <c r="M262" s="22"/>
       <c r="N262" s="5"/>
@@ -19377,15 +19365,15 @@
       <c r="H263" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I263" s="25" t="str">
+      <c r="I263" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J263" s="26" t="str">
+      <c r="J263" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K263" s="26"/>
+      <c r="K263" s="5"/>
       <c r="L263" s="21"/>
       <c r="M263" s="22"/>
       <c r="N263" s="5"/>
@@ -19419,15 +19407,15 @@
       <c r="H264" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I264" s="25" t="str">
+      <c r="I264" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J264" s="26" t="str">
+      <c r="J264" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K264" s="26"/>
+      <c r="K264" s="5"/>
       <c r="L264" s="21"/>
       <c r="M264" s="22"/>
       <c r="N264" s="5"/>
@@ -19461,15 +19449,15 @@
       <c r="H265" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I265" s="25" t="str">
+      <c r="I265" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J265" s="26" t="str">
+      <c r="J265" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K265" s="26"/>
+      <c r="K265" s="5"/>
       <c r="L265" s="21"/>
       <c r="M265" s="22"/>
       <c r="N265" s="5"/>
@@ -19503,15 +19491,15 @@
       <c r="H266" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I266" s="25" t="str">
+      <c r="I266" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J266" s="26" t="str">
+      <c r="J266" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K266" s="26"/>
+      <c r="K266" s="5"/>
       <c r="L266" s="21"/>
       <c r="M266" s="22"/>
       <c r="N266" s="5"/>
@@ -19545,15 +19533,15 @@
       <c r="H267" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I267" s="25" t="str">
+      <c r="I267" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J267" s="26" t="str">
+      <c r="J267" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K267" s="26"/>
+      <c r="K267" s="5"/>
       <c r="L267" s="21"/>
       <c r="M267" s="22"/>
       <c r="N267" s="5"/>
@@ -19587,15 +19575,15 @@
       <c r="H268" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="I268" s="25" t="str">
+      <c r="I268" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J268" s="26" t="str">
+      <c r="J268" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K268" s="26"/>
+      <c r="K268" s="5"/>
       <c r="L268" s="21"/>
       <c r="M268" s="22"/>
       <c r="N268" s="5"/>
@@ -19629,15 +19617,15 @@
       <c r="H269" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I269" s="25" t="str">
+      <c r="I269" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J269" s="26" t="str">
+      <c r="J269" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K269" s="26"/>
+      <c r="K269" s="5"/>
       <c r="L269" s="21"/>
       <c r="M269" s="22"/>
       <c r="N269" s="5"/>
@@ -19671,15 +19659,15 @@
       <c r="H270" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I270" s="25" t="str">
+      <c r="I270" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J270" s="26" t="str">
+      <c r="J270" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K270" s="26"/>
+      <c r="K270" s="5"/>
       <c r="L270" s="21"/>
       <c r="M270" s="22"/>
       <c r="N270" s="5"/>
@@ -19713,15 +19701,15 @@
       <c r="H271" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I271" s="25" t="str">
+      <c r="I271" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J271" s="26" t="str">
+      <c r="J271" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K271" s="26"/>
+      <c r="K271" s="5"/>
       <c r="L271" s="21"/>
       <c r="M271" s="22"/>
       <c r="N271" s="5"/>
@@ -19755,15 +19743,15 @@
       <c r="H272" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I272" s="25" t="str">
+      <c r="I272" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J272" s="26" t="str">
+      <c r="J272" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K272" s="26"/>
+      <c r="K272" s="5"/>
       <c r="L272" s="21"/>
       <c r="M272" s="22"/>
       <c r="N272" s="5"/>
@@ -19797,15 +19785,15 @@
       <c r="H273" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I273" s="25" t="str">
+      <c r="I273" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J273" s="26" t="str">
+      <c r="J273" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K273" s="26"/>
+      <c r="K273" s="5"/>
       <c r="L273" s="21"/>
       <c r="M273" s="22"/>
       <c r="N273" s="5"/>
@@ -19839,15 +19827,15 @@
       <c r="H274" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I274" s="25" t="str">
+      <c r="I274" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J274" s="26" t="str">
+      <c r="J274" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K274" s="26"/>
+      <c r="K274" s="5"/>
       <c r="L274" s="21"/>
       <c r="M274" s="22"/>
       <c r="N274" s="5"/>
@@ -19881,15 +19869,15 @@
       <c r="H275" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I275" s="25" t="str">
+      <c r="I275" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J275" s="26" t="str">
+      <c r="J275" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K275" s="26"/>
+      <c r="K275" s="5"/>
       <c r="L275" s="21"/>
       <c r="M275" s="22"/>
       <c r="N275" s="5"/>
@@ -19923,15 +19911,15 @@
       <c r="H276" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="I276" s="25" t="str">
+      <c r="I276" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J276" s="26" t="str">
+      <c r="J276" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K276" s="26"/>
+      <c r="K276" s="5"/>
       <c r="L276" s="21"/>
       <c r="M276" s="22"/>
       <c r="N276" s="5"/>
@@ -19965,15 +19953,15 @@
       <c r="H277" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I277" s="25" t="str">
+      <c r="I277" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J277" s="26" t="str">
+      <c r="J277" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K277" s="26"/>
+      <c r="K277" s="5"/>
       <c r="L277" s="21"/>
       <c r="M277" s="22"/>
       <c r="N277" s="5"/>
@@ -20007,15 +19995,15 @@
       <c r="H278" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I278" s="25" t="str">
+      <c r="I278" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J278" s="26" t="str">
+      <c r="J278" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K278" s="26"/>
+      <c r="K278" s="5"/>
       <c r="L278" s="21"/>
       <c r="M278" s="22"/>
       <c r="N278" s="5"/>
@@ -20049,15 +20037,15 @@
       <c r="H279" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I279" s="25" t="str">
+      <c r="I279" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J279" s="26" t="str">
+      <c r="J279" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K279" s="26"/>
+      <c r="K279" s="5"/>
       <c r="L279" s="21"/>
       <c r="M279" s="22"/>
       <c r="N279" s="5"/>
@@ -20091,15 +20079,15 @@
       <c r="H280" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I280" s="25" t="str">
+      <c r="I280" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J280" s="26" t="str">
+      <c r="J280" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K280" s="26"/>
+      <c r="K280" s="5"/>
       <c r="L280" s="21"/>
       <c r="M280" s="22"/>
       <c r="N280" s="5"/>
@@ -20133,15 +20121,15 @@
       <c r="H281" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I281" s="25" t="str">
+      <c r="I281" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J281" s="26" t="str">
+      <c r="J281" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K281" s="26"/>
+      <c r="K281" s="5"/>
       <c r="L281" s="21"/>
       <c r="M281" s="22"/>
       <c r="N281" s="5"/>
@@ -20175,15 +20163,15 @@
       <c r="H282" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I282" s="25" t="str">
+      <c r="I282" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J282" s="26" t="str">
+      <c r="J282" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K282" s="26"/>
+      <c r="K282" s="5"/>
       <c r="L282" s="21"/>
       <c r="M282" s="22"/>
       <c r="N282" s="5"/>
@@ -20217,15 +20205,15 @@
       <c r="H283" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I283" s="25" t="str">
+      <c r="I283" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J283" s="26" t="str">
+      <c r="J283" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K283" s="26"/>
+      <c r="K283" s="5"/>
       <c r="L283" s="21"/>
       <c r="M283" s="22"/>
       <c r="N283" s="5"/>
@@ -20259,15 +20247,15 @@
       <c r="H284" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I284" s="25" t="str">
+      <c r="I284" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J284" s="26" t="str">
+      <c r="J284" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K284" s="26"/>
+      <c r="K284" s="5"/>
       <c r="L284" s="21"/>
       <c r="M284" s="22"/>
       <c r="N284" s="5"/>
@@ -20301,15 +20289,15 @@
       <c r="H285" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I285" s="25" t="str">
+      <c r="I285" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J285" s="26" t="str">
+      <c r="J285" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K285" s="26"/>
+      <c r="K285" s="5"/>
       <c r="L285" s="21"/>
       <c r="M285" s="22"/>
       <c r="N285" s="5"/>
@@ -20343,15 +20331,15 @@
       <c r="H286" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I286" s="25" t="str">
+      <c r="I286" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J286" s="26" t="str">
+      <c r="J286" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K286" s="26"/>
+      <c r="K286" s="5"/>
       <c r="L286" s="21"/>
       <c r="M286" s="22"/>
       <c r="N286" s="5"/>
@@ -20385,15 +20373,15 @@
       <c r="H287" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="I287" s="25" t="str">
+      <c r="I287" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Não</v>
       </c>
-      <c r="J287" s="26" t="str">
+      <c r="J287" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v>-</v>
       </c>
-      <c r="K287" s="26"/>
+      <c r="K287" s="5"/>
       <c r="L287" s="21"/>
       <c r="M287" s="22"/>
       <c r="N287" s="5"/>
@@ -20427,15 +20415,15 @@
       <c r="H288" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="I288" s="25" t="str">
+      <c r="I288" s="3" t="str">
         <f>IF(Tabela253[[#This Row],[Formato]]="rvt","Sim","Não")</f>
         <v>Sim</v>
       </c>
-      <c r="J288" s="26" t="str">
+      <c r="J288" s="5" t="str">
         <f>IF(Tabela253[[#This Row],[Modelo?]]="Sim"," ","-")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K288" s="26"/>
+      <c r="K288" s="5"/>
       <c r="L288" s="21"/>
       <c r="M288" s="22"/>
       <c r="N288" s="5"/>
@@ -20452,9 +20440,9 @@
       <c r="F289" s="3"/>
       <c r="G289" s="3"/>
       <c r="H289" s="3"/>
-      <c r="I289" s="25"/>
-      <c r="J289" s="26"/>
-      <c r="K289" s="26"/>
+      <c r="I289" s="3"/>
+      <c r="J289" s="5"/>
+      <c r="K289" s="5"/>
       <c r="L289" s="21"/>
       <c r="M289" s="22"/>
       <c r="N289" s="5"/>
@@ -20471,9 +20459,9 @@
       <c r="F290" s="3"/>
       <c r="G290" s="3"/>
       <c r="H290" s="3"/>
-      <c r="I290" s="25"/>
-      <c r="J290" s="26"/>
-      <c r="K290" s="26"/>
+      <c r="I290" s="3"/>
+      <c r="J290" s="5"/>
+      <c r="K290" s="5"/>
       <c r="L290" s="21"/>
       <c r="M290" s="22"/>
       <c r="N290" s="5"/>
@@ -20490,9 +20478,9 @@
       <c r="F291" s="3"/>
       <c r="G291" s="3"/>
       <c r="H291" s="3"/>
-      <c r="I291" s="25"/>
-      <c r="J291" s="26"/>
-      <c r="K291" s="26"/>
+      <c r="I291" s="3"/>
+      <c r="J291" s="5"/>
+      <c r="K291" s="5"/>
       <c r="L291" s="21"/>
       <c r="M291" s="22"/>
       <c r="N291" s="5"/>
@@ -20509,9 +20497,9 @@
       <c r="F292" s="3"/>
       <c r="G292" s="3"/>
       <c r="H292" s="3"/>
-      <c r="I292" s="25"/>
-      <c r="J292" s="26"/>
-      <c r="K292" s="26"/>
+      <c r="I292" s="3"/>
+      <c r="J292" s="5"/>
+      <c r="K292" s="5"/>
       <c r="L292" s="21"/>
       <c r="M292" s="22"/>
       <c r="N292" s="5"/>
@@ -20528,9 +20516,9 @@
       <c r="F293" s="3"/>
       <c r="G293" s="3"/>
       <c r="H293" s="3"/>
-      <c r="I293" s="25"/>
-      <c r="J293" s="26"/>
-      <c r="K293" s="26"/>
+      <c r="I293" s="3"/>
+      <c r="J293" s="5"/>
+      <c r="K293" s="5"/>
       <c r="L293" s="21"/>
       <c r="M293" s="22"/>
       <c r="N293" s="5"/>
@@ -20547,9 +20535,9 @@
       <c r="F294" s="3"/>
       <c r="G294" s="3"/>
       <c r="H294" s="3"/>
-      <c r="I294" s="25"/>
-      <c r="J294" s="26"/>
-      <c r="K294" s="26"/>
+      <c r="I294" s="3"/>
+      <c r="J294" s="5"/>
+      <c r="K294" s="5"/>
       <c r="L294" s="21"/>
       <c r="M294" s="22"/>
       <c r="N294" s="5"/>
@@ -20566,9 +20554,9 @@
       <c r="F295" s="3"/>
       <c r="G295" s="3"/>
       <c r="H295" s="3"/>
-      <c r="I295" s="25"/>
-      <c r="J295" s="26"/>
-      <c r="K295" s="26"/>
+      <c r="I295" s="3"/>
+      <c r="J295" s="5"/>
+      <c r="K295" s="5"/>
       <c r="L295" s="21"/>
       <c r="M295" s="22"/>
       <c r="N295" s="5"/>
@@ -20585,9 +20573,9 @@
       <c r="F296" s="3"/>
       <c r="G296" s="3"/>
       <c r="H296" s="3"/>
-      <c r="I296" s="25"/>
-      <c r="J296" s="26"/>
-      <c r="K296" s="26"/>
+      <c r="I296" s="3"/>
+      <c r="J296" s="5"/>
+      <c r="K296" s="5"/>
       <c r="L296" s="21"/>
       <c r="M296" s="22"/>
       <c r="N296" s="5"/>
@@ -20604,9 +20592,9 @@
       <c r="F297" s="3"/>
       <c r="G297" s="3"/>
       <c r="H297" s="3"/>
-      <c r="I297" s="25"/>
-      <c r="J297" s="26"/>
-      <c r="K297" s="26"/>
+      <c r="I297" s="3"/>
+      <c r="J297" s="5"/>
+      <c r="K297" s="5"/>
       <c r="L297" s="21"/>
       <c r="M297" s="22"/>
       <c r="N297" s="5"/>
@@ -20623,9 +20611,9 @@
       <c r="F298" s="3"/>
       <c r="G298" s="3"/>
       <c r="H298" s="3"/>
-      <c r="I298" s="25"/>
-      <c r="J298" s="26"/>
-      <c r="K298" s="26"/>
+      <c r="I298" s="3"/>
+      <c r="J298" s="5"/>
+      <c r="K298" s="5"/>
       <c r="L298" s="21"/>
       <c r="M298" s="22"/>
       <c r="N298" s="5"/>
@@ -20642,9 +20630,9 @@
       <c r="F299" s="3"/>
       <c r="G299" s="3"/>
       <c r="H299" s="3"/>
-      <c r="I299" s="25"/>
-      <c r="J299" s="26"/>
-      <c r="K299" s="26"/>
+      <c r="I299" s="3"/>
+      <c r="J299" s="5"/>
+      <c r="K299" s="5"/>
       <c r="L299" s="21"/>
       <c r="M299" s="22"/>
       <c r="N299" s="5"/>
@@ -20661,9 +20649,9 @@
       <c r="F300" s="3"/>
       <c r="G300" s="3"/>
       <c r="H300" s="3"/>
-      <c r="I300" s="25"/>
-      <c r="J300" s="26"/>
-      <c r="K300" s="26"/>
+      <c r="I300" s="3"/>
+      <c r="J300" s="5"/>
+      <c r="K300" s="5"/>
       <c r="L300" s="21"/>
       <c r="M300" s="22"/>
       <c r="N300" s="5"/>
@@ -20680,9 +20668,9 @@
       <c r="F301" s="3"/>
       <c r="G301" s="3"/>
       <c r="H301" s="3"/>
-      <c r="I301" s="25"/>
-      <c r="J301" s="26"/>
-      <c r="K301" s="26"/>
+      <c r="I301" s="3"/>
+      <c r="J301" s="5"/>
+      <c r="K301" s="5"/>
       <c r="L301" s="21"/>
       <c r="M301" s="22"/>
       <c r="N301" s="5"/>
@@ -20699,9 +20687,9 @@
       <c r="F302" s="3"/>
       <c r="G302" s="3"/>
       <c r="H302" s="3"/>
-      <c r="I302" s="25"/>
-      <c r="J302" s="26"/>
-      <c r="K302" s="26"/>
+      <c r="I302" s="3"/>
+      <c r="J302" s="5"/>
+      <c r="K302" s="5"/>
       <c r="L302" s="21"/>
       <c r="M302" s="22"/>
       <c r="N302" s="5"/>
@@ -20718,9 +20706,9 @@
       <c r="F303" s="3"/>
       <c r="G303" s="3"/>
       <c r="H303" s="3"/>
-      <c r="I303" s="25"/>
-      <c r="J303" s="26"/>
-      <c r="K303" s="26"/>
+      <c r="I303" s="3"/>
+      <c r="J303" s="5"/>
+      <c r="K303" s="5"/>
       <c r="L303" s="21"/>
       <c r="M303" s="22"/>
       <c r="N303" s="5"/>
@@ -20737,9 +20725,9 @@
       <c r="F304" s="3"/>
       <c r="G304" s="3"/>
       <c r="H304" s="3"/>
-      <c r="I304" s="25"/>
-      <c r="J304" s="26"/>
-      <c r="K304" s="26"/>
+      <c r="I304" s="3"/>
+      <c r="J304" s="5"/>
+      <c r="K304" s="5"/>
       <c r="L304" s="21"/>
       <c r="M304" s="22"/>
       <c r="N304" s="5"/>
@@ -20756,9 +20744,9 @@
       <c r="F305" s="3"/>
       <c r="G305" s="3"/>
       <c r="H305" s="3"/>
-      <c r="I305" s="25"/>
-      <c r="J305" s="26"/>
-      <c r="K305" s="26"/>
+      <c r="I305" s="3"/>
+      <c r="J305" s="5"/>
+      <c r="K305" s="5"/>
       <c r="L305" s="21"/>
       <c r="M305" s="22"/>
       <c r="N305" s="5"/>
@@ -20775,9 +20763,9 @@
       <c r="F306" s="3"/>
       <c r="G306" s="3"/>
       <c r="H306" s="3"/>
-      <c r="I306" s="25"/>
-      <c r="J306" s="26"/>
-      <c r="K306" s="26"/>
+      <c r="I306" s="3"/>
+      <c r="J306" s="5"/>
+      <c r="K306" s="5"/>
       <c r="L306" s="21"/>
       <c r="M306" s="22"/>
       <c r="N306" s="5"/>
@@ -20794,9 +20782,9 @@
       <c r="F307" s="3"/>
       <c r="G307" s="3"/>
       <c r="H307" s="3"/>
-      <c r="I307" s="25"/>
-      <c r="J307" s="26"/>
-      <c r="K307" s="26"/>
+      <c r="I307" s="3"/>
+      <c r="J307" s="5"/>
+      <c r="K307" s="5"/>
       <c r="L307" s="21"/>
       <c r="M307" s="22"/>
       <c r="N307" s="5"/>
@@ -20813,9 +20801,9 @@
       <c r="F308" s="3"/>
       <c r="G308" s="3"/>
       <c r="H308" s="3"/>
-      <c r="I308" s="25"/>
-      <c r="J308" s="26"/>
-      <c r="K308" s="26"/>
+      <c r="I308" s="3"/>
+      <c r="J308" s="5"/>
+      <c r="K308" s="5"/>
       <c r="L308" s="21"/>
       <c r="M308" s="22"/>
       <c r="N308" s="5"/>
@@ -20832,9 +20820,9 @@
       <c r="F309" s="3"/>
       <c r="G309" s="3"/>
       <c r="H309" s="3"/>
-      <c r="I309" s="25"/>
-      <c r="J309" s="26"/>
-      <c r="K309" s="26"/>
+      <c r="I309" s="3"/>
+      <c r="J309" s="5"/>
+      <c r="K309" s="5"/>
       <c r="L309" s="21"/>
       <c r="M309" s="22"/>
       <c r="N309" s="5"/>
@@ -20851,9 +20839,9 @@
       <c r="F310" s="3"/>
       <c r="G310" s="3"/>
       <c r="H310" s="3"/>
-      <c r="I310" s="25"/>
-      <c r="J310" s="26"/>
-      <c r="K310" s="26"/>
+      <c r="I310" s="3"/>
+      <c r="J310" s="5"/>
+      <c r="K310" s="5"/>
       <c r="L310" s="21"/>
       <c r="M310" s="22"/>
       <c r="N310" s="5"/>
@@ -20870,9 +20858,9 @@
       <c r="F311" s="3"/>
       <c r="G311" s="3"/>
       <c r="H311" s="3"/>
-      <c r="I311" s="25"/>
-      <c r="J311" s="26"/>
-      <c r="K311" s="26"/>
+      <c r="I311" s="3"/>
+      <c r="J311" s="5"/>
+      <c r="K311" s="5"/>
       <c r="L311" s="21"/>
       <c r="M311" s="22"/>
       <c r="N311" s="5"/>
@@ -20889,9 +20877,9 @@
       <c r="F312" s="3"/>
       <c r="G312" s="3"/>
       <c r="H312" s="3"/>
-      <c r="I312" s="25"/>
-      <c r="J312" s="26"/>
-      <c r="K312" s="26"/>
+      <c r="I312" s="3"/>
+      <c r="J312" s="5"/>
+      <c r="K312" s="5"/>
       <c r="L312" s="21"/>
       <c r="M312" s="22"/>
       <c r="N312" s="5"/>
@@ -20908,9 +20896,9 @@
       <c r="F313" s="3"/>
       <c r="G313" s="3"/>
       <c r="H313" s="3"/>
-      <c r="I313" s="25"/>
-      <c r="J313" s="26"/>
-      <c r="K313" s="26"/>
+      <c r="I313" s="3"/>
+      <c r="J313" s="5"/>
+      <c r="K313" s="5"/>
       <c r="L313" s="21"/>
       <c r="M313" s="22"/>
       <c r="N313" s="5"/>
@@ -20927,9 +20915,9 @@
       <c r="F314" s="3"/>
       <c r="G314" s="3"/>
       <c r="H314" s="3"/>
-      <c r="I314" s="25"/>
-      <c r="J314" s="26"/>
-      <c r="K314" s="26"/>
+      <c r="I314" s="3"/>
+      <c r="J314" s="5"/>
+      <c r="K314" s="5"/>
       <c r="L314" s="21"/>
       <c r="M314" s="22"/>
       <c r="N314" s="5"/>
@@ -20946,9 +20934,9 @@
       <c r="F315" s="3"/>
       <c r="G315" s="3"/>
       <c r="H315" s="3"/>
-      <c r="I315" s="25"/>
-      <c r="J315" s="26"/>
-      <c r="K315" s="26"/>
+      <c r="I315" s="3"/>
+      <c r="J315" s="5"/>
+      <c r="K315" s="5"/>
       <c r="L315" s="21"/>
       <c r="M315" s="22"/>
       <c r="N315" s="5"/>
@@ -20965,9 +20953,9 @@
       <c r="F316" s="3"/>
       <c r="G316" s="3"/>
       <c r="H316" s="3"/>
-      <c r="I316" s="25"/>
-      <c r="J316" s="26"/>
-      <c r="K316" s="26"/>
+      <c r="I316" s="3"/>
+      <c r="J316" s="5"/>
+      <c r="K316" s="5"/>
       <c r="L316" s="21"/>
       <c r="M316" s="22"/>
       <c r="N316" s="5"/>
@@ -20984,9 +20972,9 @@
       <c r="F317" s="3"/>
       <c r="G317" s="3"/>
       <c r="H317" s="3"/>
-      <c r="I317" s="25"/>
-      <c r="J317" s="26"/>
-      <c r="K317" s="26"/>
+      <c r="I317" s="3"/>
+      <c r="J317" s="5"/>
+      <c r="K317" s="5"/>
       <c r="L317" s="21"/>
       <c r="M317" s="22"/>
       <c r="N317" s="5"/>
@@ -21003,9 +20991,9 @@
       <c r="F318" s="3"/>
       <c r="G318" s="3"/>
       <c r="H318" s="3"/>
-      <c r="I318" s="25"/>
-      <c r="J318" s="26"/>
-      <c r="K318" s="26"/>
+      <c r="I318" s="3"/>
+      <c r="J318" s="5"/>
+      <c r="K318" s="5"/>
       <c r="L318" s="21"/>
       <c r="M318" s="22"/>
       <c r="N318" s="5"/>
@@ -21022,9 +21010,9 @@
       <c r="F319" s="3"/>
       <c r="G319" s="3"/>
       <c r="H319" s="3"/>
-      <c r="I319" s="25"/>
-      <c r="J319" s="26"/>
-      <c r="K319" s="26"/>
+      <c r="I319" s="3"/>
+      <c r="J319" s="5"/>
+      <c r="K319" s="5"/>
       <c r="L319" s="21"/>
       <c r="M319" s="22"/>
       <c r="N319" s="5"/>
@@ -21041,9 +21029,9 @@
       <c r="F320" s="3"/>
       <c r="G320" s="3"/>
       <c r="H320" s="3"/>
-      <c r="I320" s="25"/>
-      <c r="J320" s="26"/>
-      <c r="K320" s="26"/>
+      <c r="I320" s="3"/>
+      <c r="J320" s="5"/>
+      <c r="K320" s="5"/>
       <c r="L320" s="21"/>
       <c r="M320" s="22"/>
       <c r="N320" s="5"/>
@@ -21060,9 +21048,9 @@
       <c r="F321" s="3"/>
       <c r="G321" s="3"/>
       <c r="H321" s="3"/>
-      <c r="I321" s="25"/>
-      <c r="J321" s="26"/>
-      <c r="K321" s="26"/>
+      <c r="I321" s="3"/>
+      <c r="J321" s="5"/>
+      <c r="K321" s="5"/>
       <c r="L321" s="21"/>
       <c r="M321" s="22"/>
       <c r="N321" s="5"/>
@@ -21079,9 +21067,9 @@
       <c r="F322" s="3"/>
       <c r="G322" s="3"/>
       <c r="H322" s="3"/>
-      <c r="I322" s="25"/>
-      <c r="J322" s="26"/>
-      <c r="K322" s="26"/>
+      <c r="I322" s="3"/>
+      <c r="J322" s="5"/>
+      <c r="K322" s="5"/>
       <c r="L322" s="21"/>
       <c r="M322" s="22"/>
       <c r="N322" s="5"/>
@@ -21098,9 +21086,9 @@
       <c r="F323" s="3"/>
       <c r="G323" s="3"/>
       <c r="H323" s="3"/>
-      <c r="I323" s="25"/>
-      <c r="J323" s="26"/>
-      <c r="K323" s="26"/>
+      <c r="I323" s="3"/>
+      <c r="J323" s="5"/>
+      <c r="K323" s="5"/>
       <c r="L323" s="21"/>
       <c r="M323" s="22"/>
       <c r="N323" s="5"/>
@@ -21117,9 +21105,9 @@
       <c r="F324" s="3"/>
       <c r="G324" s="3"/>
       <c r="H324" s="3"/>
-      <c r="I324" s="25"/>
-      <c r="J324" s="26"/>
-      <c r="K324" s="26"/>
+      <c r="I324" s="3"/>
+      <c r="J324" s="5"/>
+      <c r="K324" s="5"/>
       <c r="L324" s="21"/>
       <c r="M324" s="22"/>
       <c r="N324" s="5"/>
@@ -21136,9 +21124,9 @@
       <c r="F325" s="3"/>
       <c r="G325" s="3"/>
       <c r="H325" s="3"/>
-      <c r="I325" s="25"/>
-      <c r="J325" s="26"/>
-      <c r="K325" s="26"/>
+      <c r="I325" s="3"/>
+      <c r="J325" s="5"/>
+      <c r="K325" s="5"/>
       <c r="L325" s="21"/>
       <c r="M325" s="22"/>
       <c r="N325" s="5"/>
@@ -21155,9 +21143,9 @@
       <c r="F326" s="3"/>
       <c r="G326" s="3"/>
       <c r="H326" s="3"/>
-      <c r="I326" s="25"/>
-      <c r="J326" s="26"/>
-      <c r="K326" s="26"/>
+      <c r="I326" s="3"/>
+      <c r="J326" s="5"/>
+      <c r="K326" s="5"/>
       <c r="L326" s="21"/>
       <c r="M326" s="22"/>
       <c r="N326" s="5"/>
@@ -21174,9 +21162,9 @@
       <c r="F327" s="3"/>
       <c r="G327" s="3"/>
       <c r="H327" s="3"/>
-      <c r="I327" s="25"/>
-      <c r="J327" s="26"/>
-      <c r="K327" s="26"/>
+      <c r="I327" s="3"/>
+      <c r="J327" s="5"/>
+      <c r="K327" s="5"/>
       <c r="L327" s="21"/>
       <c r="M327" s="22"/>
       <c r="N327" s="5"/>
@@ -21193,9 +21181,9 @@
       <c r="F328" s="3"/>
       <c r="G328" s="3"/>
       <c r="H328" s="3"/>
-      <c r="I328" s="25"/>
-      <c r="J328" s="26"/>
-      <c r="K328" s="26"/>
+      <c r="I328" s="3"/>
+      <c r="J328" s="5"/>
+      <c r="K328" s="5"/>
       <c r="L328" s="21"/>
       <c r="M328" s="22"/>
       <c r="N328" s="5"/>
@@ -21212,9 +21200,9 @@
       <c r="F329" s="3"/>
       <c r="G329" s="3"/>
       <c r="H329" s="3"/>
-      <c r="I329" s="25"/>
-      <c r="J329" s="26"/>
-      <c r="K329" s="26"/>
+      <c r="I329" s="3"/>
+      <c r="J329" s="5"/>
+      <c r="K329" s="5"/>
       <c r="L329" s="21"/>
       <c r="M329" s="22"/>
       <c r="N329" s="5"/>
@@ -21231,9 +21219,9 @@
       <c r="F330" s="3"/>
       <c r="G330" s="3"/>
       <c r="H330" s="3"/>
-      <c r="I330" s="25"/>
-      <c r="J330" s="26"/>
-      <c r="K330" s="26"/>
+      <c r="I330" s="3"/>
+      <c r="J330" s="5"/>
+      <c r="K330" s="5"/>
       <c r="L330" s="21"/>
       <c r="M330" s="22"/>
       <c r="N330" s="5"/>
@@ -21250,9 +21238,9 @@
       <c r="F331" s="3"/>
       <c r="G331" s="3"/>
       <c r="H331" s="3"/>
-      <c r="I331" s="25"/>
-      <c r="J331" s="26"/>
-      <c r="K331" s="26"/>
+      <c r="I331" s="3"/>
+      <c r="J331" s="5"/>
+      <c r="K331" s="5"/>
       <c r="L331" s="21"/>
       <c r="M331" s="22"/>
       <c r="N331" s="5"/>
@@ -21269,9 +21257,9 @@
       <c r="F332" s="12"/>
       <c r="G332" s="12"/>
       <c r="H332" s="12"/>
-      <c r="I332" s="27"/>
-      <c r="J332" s="28"/>
-      <c r="K332" s="28"/>
+      <c r="I332" s="12"/>
+      <c r="J332" s="14"/>
+      <c r="K332" s="14"/>
       <c r="L332" s="23"/>
       <c r="M332" s="24"/>
       <c r="N332" s="14"/>
@@ -21281,23 +21269,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J182:J183 N2 P2:Q2 N3:Q234">
-    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"-"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K36:K37 K57:K58 K189:K234 K65:K66 K72 K74:K75 K90 K96 K101 K107:K109 K113 K118 K123 K125:K127 K137 K140 K150:K187">
-    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="PENDENTE">
+  <conditionalFormatting sqref="K36:K37 K57:K58 K65:K66 K72 K74:K75 K90 K96 K101 K107:K109 K113 K118 K123 K125:K127 K137 K140 K150:K187 K189:K234">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="PENDENTE">
       <formula>NOT(ISERROR(SEARCH("PENDENTE",K36)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="5" operator="containsText" text="LIBERADO">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="LIBERADO">
       <formula>NOT(ISERROR(SEARCH("LIBERADO",K36)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M16 M164 M181 M198 M210 M223">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="6" operator="equal">
       <formula>"Não"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="7" operator="equal">
       <formula>"Sim"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat: ajusta mapeamento de entregas As-Built e adiciona script de importacao final
</commit_message>
<xml_diff>
--- a/Planilhas/Mapeamento Modelos As Built.xlsx
+++ b/Planilhas/Mapeamento Modelos As Built.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\STECLA IA\Dashboard-AsBuilt-Custom\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RenataViannaKüster\Downloads\01.Neodent\8. As built\Entregas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940680D8-86BA-4AD2-B2B4-A2F3ECCCF6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF671178-E914-4970-8E06-AA43646749C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{01155B47-A7E1-4A45-B27D-D246D4740F40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{01155B47-A7E1-4A45-B27D-D246D4740F40}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapeamento Modelos As Built" sheetId="1" r:id="rId1"/>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2765" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2935" uniqueCount="672">
   <si>
     <t>Número</t>
   </si>
@@ -2009,6 +2009,114 @@
   </si>
   <si>
     <t>NEO-23001-AS-ELE-001-MOD PRODUCAO 19.03-R08</t>
+  </si>
+  <si>
+    <t>008. SM 61 - 06.04.2026</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-16-HID-MO-001-R23</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-PAV-001-PAVIM-R01</t>
+  </si>
+  <si>
+    <t>SPN.ARQ.00.AS.001.R05-Implantação Geral</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Instalações Hidráulicas</t>
+  </si>
+  <si>
+    <t>Modelo do predio produção, mas atualizaram as caixas. Precisa atualizar no modelo de estrutura ( Alteração na posição das caixas hidráulicas 9 (Execuatda - POSTADO)). Este modelos é o do predio produção. Vamos manter como Predio Produção</t>
+  </si>
+  <si>
+    <t>Estava descoordenado. Stecla ajustou. Pavimentação do patio e central de utilidades não tem. Será feito em entrega posterior? Nível da pavimentação Sede Recreativa não está compatível com projeto (mesmo nível do prédio suporte). Será atualizado em entrega posterior? Calçada do eixo A não acompanha desnível do terreno</t>
+  </si>
+  <si>
+    <t>Está igual ao modelo de pavimentação - qual sonsiderar?</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-00-ARQ-MO-PROD1-R08</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-16-HID-MO-002-R19</t>
+  </si>
+  <si>
+    <t>SPN.ARQ.02.AS.002.003.004.R08-Planta 2 Pav (SETORES A-B-C)</t>
+  </si>
+  <si>
+    <t>SPN.ARQ.02.AS.005.006.007.R08-Planta 3 Pav (SETORES A-B-C)</t>
+  </si>
+  <si>
+    <t>SPN.ARQ.02.AS.008.009.010.R08-Planta 4 Pav (SETORES A-B-C)</t>
+  </si>
+  <si>
+    <t>Modelo dos isopainéis. Não está coordendado com coordenadas compartilhadas - Stecla ajustou. Há painéis voando no modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construção de shaft - Vest. Fem. 2º pvto </t>
+  </si>
+  <si>
+    <t>Mudança na Posição /Diminuição de esquadria no 3º pvto - Sala Controlada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alteração no layout da área "Reserva" no 4º pvto do Prédio de Produção </t>
+  </si>
+  <si>
+    <t>modelo de agua fria - não estava na planilha de controle de entregas. Foram feitos alguns ajustes de tubulações, mas ainda não refletem ao que foi realmente executado (Microbiologia e TNC)</t>
+  </si>
+  <si>
+    <t>03. SM 13 - 25.03.2026 ETE</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-ELE-001-INFRA 25.03-R00</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-HID-001-INFRA 25.03-R00</t>
+  </si>
+  <si>
+    <t>04. SM 15 - 08.04.2026 ETE</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-HID-001-INFRA 08.04-R00</t>
+  </si>
+  <si>
+    <t>023. SM 14 - 02.04.2026</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-ELE-001-MOD PRODUCAO 02.04-R08</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-BAR-001-MOD 02.04-R03</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-LOG-001-MOD PRODUCAO 02.04-R01</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-16-PCI HID-MO-001-02.04.26-R16</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-PCI-MO-002-SPRINKLER 02.04.26-R17</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-CLI 02.04-000-R18</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-17-UTI-MO 02.04-001-R25</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-SDA-003-MOD PRODUCAO 02.04.26-R04</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-AUT-002-MOD-PRODUCAO 02.04-R02</t>
+  </si>
+  <si>
+    <t>NEO-23001-AS-AUT-005-MOD-UTILIDADES 02.04-R00</t>
   </si>
 </sst>
 </file>
@@ -8066,8 +8174,8 @@
     <col min="7" max="7" width="81.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" style="18" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="44.28515625" style="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.28515625" style="18" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="32.7109375" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="91.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="66.42578125" style="18" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="33" bestFit="1" customWidth="1"/>
@@ -20520,44 +20628,80 @@
       <c r="P290" s="8"/>
       <c r="Q290" s="8"/>
     </row>
-    <row r="291" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A291" s="3">
         <f t="shared" si="3"/>
         <v>290</v>
       </c>
-      <c r="B291" s="3"/>
-      <c r="C291" s="3"/>
-      <c r="D291" s="3"/>
-      <c r="E291" s="3"/>
-      <c r="F291" s="3"/>
-      <c r="G291" s="3"/>
-      <c r="H291" s="3"/>
-      <c r="I291" s="3"/>
+      <c r="B291" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C291" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D291" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E291" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F291" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="G291" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="H291" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I291" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J291" s="5"/>
       <c r="K291" s="5"/>
-      <c r="L291" s="21"/>
+      <c r="L291" s="21" t="s">
+        <v>642</v>
+      </c>
       <c r="M291" s="22"/>
       <c r="N291" s="5"/>
       <c r="O291" s="17"/>
       <c r="P291" s="8"/>
       <c r="Q291" s="8"/>
     </row>
-    <row r="292" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A292" s="3">
         <f t="shared" si="3"/>
         <v>291</v>
       </c>
-      <c r="B292" s="3"/>
-      <c r="C292" s="3"/>
-      <c r="D292" s="3"/>
-      <c r="E292" s="3"/>
-      <c r="F292" s="3"/>
-      <c r="G292" s="3"/>
-      <c r="H292" s="3"/>
-      <c r="I292" s="3"/>
+      <c r="B292" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D292" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E292" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G292" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="H292" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I292" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J292" s="5"/>
       <c r="K292" s="5"/>
-      <c r="L292" s="21"/>
+      <c r="L292" s="21" t="s">
+        <v>643</v>
+      </c>
       <c r="M292" s="22"/>
       <c r="N292" s="5"/>
       <c r="O292" s="17"/>
@@ -20569,14 +20713,30 @@
         <f t="shared" si="3"/>
         <v>292</v>
       </c>
-      <c r="B293" s="3"/>
-      <c r="C293" s="3"/>
-      <c r="D293" s="3"/>
-      <c r="E293" s="3"/>
-      <c r="F293" s="3"/>
-      <c r="G293" s="3"/>
-      <c r="H293" s="3"/>
-      <c r="I293" s="3"/>
+      <c r="B293" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C293" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D293" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E293" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F293" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G293" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="H293" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="I293" s="3" t="s">
+        <v>640</v>
+      </c>
       <c r="J293" s="5"/>
       <c r="K293" s="5"/>
       <c r="L293" s="21"/>
@@ -20591,61 +20751,111 @@
         <f t="shared" si="3"/>
         <v>293</v>
       </c>
-      <c r="B294" s="3"/>
-      <c r="C294" s="3"/>
-      <c r="D294" s="3"/>
-      <c r="E294" s="3"/>
-      <c r="F294" s="3"/>
-      <c r="G294" s="3"/>
-      <c r="H294" s="3"/>
-      <c r="I294" s="3"/>
+      <c r="B294" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D294" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E294" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G294" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="H294" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I294" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J294" s="5"/>
       <c r="K294" s="5"/>
-      <c r="L294" s="21"/>
+      <c r="L294" s="21" t="s">
+        <v>644</v>
+      </c>
       <c r="M294" s="22"/>
       <c r="N294" s="5"/>
       <c r="O294" s="17"/>
       <c r="P294" s="8"/>
       <c r="Q294" s="8"/>
     </row>
-    <row r="295" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A295" s="3">
         <f t="shared" si="3"/>
         <v>294</v>
       </c>
-      <c r="B295" s="3"/>
-      <c r="C295" s="3"/>
-      <c r="D295" s="3"/>
-      <c r="E295" s="3"/>
-      <c r="F295" s="3"/>
-      <c r="G295" s="3"/>
-      <c r="H295" s="3"/>
+      <c r="B295" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E295" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F295" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G295" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="H295" s="3" t="s">
+        <v>291</v>
+      </c>
       <c r="I295" s="3"/>
       <c r="J295" s="5"/>
       <c r="K295" s="5"/>
-      <c r="L295" s="21"/>
+      <c r="L295" s="21" t="s">
+        <v>650</v>
+      </c>
       <c r="M295" s="22"/>
       <c r="N295" s="5"/>
       <c r="O295" s="17"/>
       <c r="P295" s="8"/>
       <c r="Q295" s="8"/>
     </row>
-    <row r="296" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A296" s="3">
         <f t="shared" si="3"/>
         <v>295</v>
       </c>
-      <c r="B296" s="3"/>
-      <c r="C296" s="3"/>
-      <c r="D296" s="3"/>
-      <c r="E296" s="3"/>
+      <c r="B296" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D296" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E296" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="F296" s="3"/>
-      <c r="G296" s="3"/>
-      <c r="H296" s="3"/>
-      <c r="I296" s="3"/>
+      <c r="G296" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="H296" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I296" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J296" s="5"/>
       <c r="K296" s="5"/>
-      <c r="L296" s="21"/>
+      <c r="L296" s="21" t="s">
+        <v>654</v>
+      </c>
       <c r="M296" s="22"/>
       <c r="N296" s="5"/>
       <c r="O296" s="17"/>
@@ -20657,17 +20867,35 @@
         <f t="shared" si="3"/>
         <v>296</v>
       </c>
-      <c r="B297" s="3"/>
-      <c r="C297" s="3"/>
-      <c r="D297" s="3"/>
-      <c r="E297" s="3"/>
-      <c r="F297" s="3"/>
-      <c r="G297" s="3"/>
-      <c r="H297" s="3"/>
-      <c r="I297" s="3"/>
+      <c r="B297" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D297" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E297" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F297" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G297" s="3" t="s">
+        <v>647</v>
+      </c>
+      <c r="H297" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="I297" s="3" t="s">
+        <v>640</v>
+      </c>
       <c r="J297" s="5"/>
       <c r="K297" s="5"/>
-      <c r="L297" s="21"/>
+      <c r="L297" s="21" t="s">
+        <v>651</v>
+      </c>
       <c r="M297" s="22"/>
       <c r="N297" s="5"/>
       <c r="O297" s="17"/>
@@ -20679,17 +20907,35 @@
         <f t="shared" si="3"/>
         <v>297</v>
       </c>
-      <c r="B298" s="3"/>
-      <c r="C298" s="3"/>
-      <c r="D298" s="3"/>
-      <c r="E298" s="3"/>
-      <c r="F298" s="3"/>
-      <c r="G298" s="3"/>
-      <c r="H298" s="3"/>
-      <c r="I298" s="3"/>
+      <c r="B298" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D298" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E298" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F298" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G298" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="H298" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="I298" s="3" t="s">
+        <v>640</v>
+      </c>
       <c r="J298" s="5"/>
       <c r="K298" s="5"/>
-      <c r="L298" s="21"/>
+      <c r="L298" s="21" t="s">
+        <v>652</v>
+      </c>
       <c r="M298" s="22"/>
       <c r="N298" s="5"/>
       <c r="O298" s="17"/>
@@ -20701,17 +20947,35 @@
         <f t="shared" si="3"/>
         <v>298</v>
       </c>
-      <c r="B299" s="3"/>
-      <c r="C299" s="3"/>
-      <c r="D299" s="3"/>
-      <c r="E299" s="3"/>
-      <c r="F299" s="3"/>
-      <c r="G299" s="3"/>
-      <c r="H299" s="3"/>
-      <c r="I299" s="3"/>
+      <c r="B299" s="8">
+        <v>46118</v>
+      </c>
+      <c r="C299" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="D299" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E299" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F299" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G299" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="H299" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="I299" s="3" t="s">
+        <v>640</v>
+      </c>
       <c r="J299" s="5"/>
       <c r="K299" s="5"/>
-      <c r="L299" s="21"/>
+      <c r="L299" s="21" t="s">
+        <v>653</v>
+      </c>
       <c r="M299" s="22"/>
       <c r="N299" s="5"/>
       <c r="O299" s="17"/>
@@ -20723,14 +20987,30 @@
         <f t="shared" si="3"/>
         <v>299</v>
       </c>
-      <c r="B300" s="3"/>
-      <c r="C300" s="3"/>
-      <c r="D300" s="3"/>
-      <c r="E300" s="3"/>
-      <c r="F300" s="3"/>
-      <c r="G300" s="3"/>
-      <c r="H300" s="3"/>
-      <c r="I300" s="3"/>
+      <c r="B300" s="8">
+        <v>46106</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D300" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E300" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G300" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="H300" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I300" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J300" s="5"/>
       <c r="K300" s="5"/>
       <c r="L300" s="21"/>
@@ -20745,14 +21025,30 @@
         <f t="shared" si="3"/>
         <v>300</v>
       </c>
-      <c r="B301" s="3"/>
-      <c r="C301" s="3"/>
-      <c r="D301" s="3"/>
-      <c r="E301" s="3"/>
-      <c r="F301" s="3"/>
-      <c r="G301" s="3"/>
-      <c r="H301" s="3"/>
-      <c r="I301" s="3"/>
+      <c r="B301" s="8">
+        <v>46106</v>
+      </c>
+      <c r="C301" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="D301" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E301" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F301" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="G301" s="3" t="s">
+        <v>657</v>
+      </c>
+      <c r="H301" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I301" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J301" s="5"/>
       <c r="K301" s="5"/>
       <c r="L301" s="21"/>
@@ -20767,14 +21063,30 @@
         <f t="shared" si="3"/>
         <v>301</v>
       </c>
-      <c r="B302" s="3"/>
-      <c r="C302" s="3"/>
-      <c r="D302" s="3"/>
-      <c r="E302" s="3"/>
-      <c r="F302" s="3"/>
-      <c r="G302" s="3"/>
-      <c r="H302" s="3"/>
-      <c r="I302" s="3"/>
+      <c r="B302" s="8">
+        <v>46120</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="D302" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E302" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="G302" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="H302" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I302" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J302" s="5"/>
       <c r="K302" s="5"/>
       <c r="L302" s="21"/>
@@ -20789,17 +21101,35 @@
         <f t="shared" si="3"/>
         <v>302</v>
       </c>
-      <c r="B303" s="3"/>
-      <c r="C303" s="3"/>
-      <c r="D303" s="3"/>
-      <c r="E303" s="3"/>
-      <c r="F303" s="3"/>
-      <c r="G303" s="3"/>
-      <c r="H303" s="3"/>
-      <c r="I303" s="3"/>
+      <c r="B303" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C303" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D303" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E303" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F303" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G303" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="H303" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I303" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J303" s="5"/>
       <c r="K303" s="5"/>
-      <c r="L303" s="21"/>
+      <c r="L303" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M303" s="22"/>
       <c r="N303" s="5"/>
       <c r="O303" s="17"/>
@@ -20811,17 +21141,35 @@
         <f t="shared" ref="A304:A332" si="4">A303+1</f>
         <v>303</v>
       </c>
-      <c r="B304" s="3"/>
-      <c r="C304" s="3"/>
-      <c r="D304" s="3"/>
-      <c r="E304" s="3"/>
-      <c r="F304" s="3"/>
-      <c r="G304" s="3"/>
-      <c r="H304" s="3"/>
-      <c r="I304" s="3"/>
+      <c r="B304" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D304" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E304" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G304" s="3" t="s">
+        <v>662</v>
+      </c>
+      <c r="H304" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I304" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J304" s="5"/>
       <c r="K304" s="5"/>
-      <c r="L304" s="21"/>
+      <c r="L304" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M304" s="22"/>
       <c r="N304" s="5"/>
       <c r="O304" s="17"/>
@@ -20833,17 +21181,35 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="B305" s="3"/>
-      <c r="C305" s="3"/>
-      <c r="D305" s="3"/>
-      <c r="E305" s="3"/>
-      <c r="F305" s="3"/>
-      <c r="G305" s="3"/>
-      <c r="H305" s="3"/>
-      <c r="I305" s="3"/>
+      <c r="B305" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C305" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D305" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E305" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F305" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G305" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="H305" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I305" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J305" s="5"/>
       <c r="K305" s="5"/>
-      <c r="L305" s="21"/>
+      <c r="L305" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M305" s="22"/>
       <c r="N305" s="5"/>
       <c r="O305" s="17"/>
@@ -20855,17 +21221,35 @@
         <f t="shared" si="4"/>
         <v>305</v>
       </c>
-      <c r="B306" s="3"/>
-      <c r="C306" s="3"/>
-      <c r="D306" s="3"/>
-      <c r="E306" s="3"/>
-      <c r="F306" s="3"/>
-      <c r="G306" s="3"/>
-      <c r="H306" s="3"/>
-      <c r="I306" s="3"/>
+      <c r="B306" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D306" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E306" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F306" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G306" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="H306" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I306" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J306" s="5"/>
       <c r="K306" s="5"/>
-      <c r="L306" s="21"/>
+      <c r="L306" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M306" s="22"/>
       <c r="N306" s="5"/>
       <c r="O306" s="17"/>
@@ -20877,17 +21261,35 @@
         <f t="shared" si="4"/>
         <v>306</v>
       </c>
-      <c r="B307" s="3"/>
-      <c r="C307" s="3"/>
-      <c r="D307" s="3"/>
-      <c r="E307" s="3"/>
-      <c r="F307" s="3"/>
-      <c r="G307" s="3"/>
-      <c r="H307" s="3"/>
-      <c r="I307" s="3"/>
+      <c r="B307" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C307" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D307" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E307" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F307" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G307" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="H307" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I307" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J307" s="5"/>
       <c r="K307" s="5"/>
-      <c r="L307" s="21"/>
+      <c r="L307" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M307" s="22"/>
       <c r="N307" s="5"/>
       <c r="O307" s="17"/>
@@ -20899,17 +21301,35 @@
         <f t="shared" si="4"/>
         <v>307</v>
       </c>
-      <c r="B308" s="3"/>
-      <c r="C308" s="3"/>
-      <c r="D308" s="3"/>
-      <c r="E308" s="3"/>
-      <c r="F308" s="3"/>
-      <c r="G308" s="3"/>
-      <c r="H308" s="3"/>
-      <c r="I308" s="3"/>
+      <c r="B308" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D308" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E308" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F308" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G308" s="3" t="s">
+        <v>667</v>
+      </c>
+      <c r="H308" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I308" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J308" s="5"/>
       <c r="K308" s="5"/>
-      <c r="L308" s="21"/>
+      <c r="L308" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M308" s="22"/>
       <c r="N308" s="5"/>
       <c r="O308" s="17"/>
@@ -20921,17 +21341,35 @@
         <f t="shared" si="4"/>
         <v>308</v>
       </c>
-      <c r="B309" s="3"/>
-      <c r="C309" s="3"/>
-      <c r="D309" s="3"/>
-      <c r="E309" s="3"/>
-      <c r="F309" s="3"/>
-      <c r="G309" s="3"/>
-      <c r="H309" s="3"/>
-      <c r="I309" s="3"/>
+      <c r="B309" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C309" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D309" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E309" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F309" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G309" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="H309" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I309" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J309" s="5"/>
       <c r="K309" s="5"/>
-      <c r="L309" s="21"/>
+      <c r="L309" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M309" s="22"/>
       <c r="N309" s="5"/>
       <c r="O309" s="17"/>
@@ -20943,17 +21381,35 @@
         <f t="shared" si="4"/>
         <v>309</v>
       </c>
-      <c r="B310" s="3"/>
-      <c r="C310" s="3"/>
-      <c r="D310" s="3"/>
-      <c r="E310" s="3"/>
-      <c r="F310" s="3"/>
-      <c r="G310" s="3"/>
-      <c r="H310" s="3"/>
-      <c r="I310" s="3"/>
+      <c r="B310" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D310" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E310" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F310" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G310" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="H310" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I310" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J310" s="5"/>
       <c r="K310" s="5"/>
-      <c r="L310" s="21"/>
+      <c r="L310" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M310" s="22"/>
       <c r="N310" s="5"/>
       <c r="O310" s="17"/>
@@ -20965,17 +21421,35 @@
         <f t="shared" si="4"/>
         <v>310</v>
       </c>
-      <c r="B311" s="3"/>
-      <c r="C311" s="3"/>
-      <c r="D311" s="3"/>
-      <c r="E311" s="3"/>
-      <c r="F311" s="3"/>
-      <c r="G311" s="3"/>
-      <c r="H311" s="3"/>
-      <c r="I311" s="3"/>
+      <c r="B311" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C311" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D311" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E311" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F311" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G311" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="H311" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I311" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J311" s="5"/>
       <c r="K311" s="5"/>
-      <c r="L311" s="21"/>
+      <c r="L311" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M311" s="22"/>
       <c r="N311" s="5"/>
       <c r="O311" s="17"/>
@@ -20987,17 +21461,35 @@
         <f t="shared" si="4"/>
         <v>311</v>
       </c>
-      <c r="B312" s="3"/>
-      <c r="C312" s="3"/>
-      <c r="D312" s="3"/>
-      <c r="E312" s="3"/>
-      <c r="F312" s="3"/>
-      <c r="G312" s="3"/>
-      <c r="H312" s="3"/>
-      <c r="I312" s="3"/>
+      <c r="B312" s="8">
+        <v>46114</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="D312" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F312" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G312" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="H312" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="I312" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J312" s="5"/>
       <c r="K312" s="5"/>
-      <c r="L312" s="21"/>
+      <c r="L312" s="21" t="s">
+        <v>663</v>
+      </c>
       <c r="M312" s="22"/>
       <c r="N312" s="5"/>
       <c r="O312" s="17"/>
@@ -21009,7 +21501,7 @@
         <f t="shared" si="4"/>
         <v>312</v>
       </c>
-      <c r="B313" s="3"/>
+      <c r="B313" s="8"/>
       <c r="C313" s="3"/>
       <c r="D313" s="3"/>
       <c r="E313" s="3"/>
@@ -21031,7 +21523,7 @@
         <f t="shared" si="4"/>
         <v>313</v>
       </c>
-      <c r="B314" s="3"/>
+      <c r="B314" s="8"/>
       <c r="C314" s="3"/>
       <c r="D314" s="3"/>
       <c r="E314" s="3"/>
@@ -21053,7 +21545,7 @@
         <f t="shared" si="4"/>
         <v>314</v>
       </c>
-      <c r="B315" s="3"/>
+      <c r="B315" s="8"/>
       <c r="C315" s="3"/>
       <c r="D315" s="3"/>
       <c r="E315" s="3"/>
@@ -21075,7 +21567,7 @@
         <f t="shared" si="4"/>
         <v>315</v>
       </c>
-      <c r="B316" s="3"/>
+      <c r="B316" s="8"/>
       <c r="C316" s="3"/>
       <c r="D316" s="3"/>
       <c r="E316" s="3"/>
@@ -21097,7 +21589,7 @@
         <f t="shared" si="4"/>
         <v>316</v>
       </c>
-      <c r="B317" s="3"/>
+      <c r="B317" s="8"/>
       <c r="C317" s="3"/>
       <c r="D317" s="3"/>
       <c r="E317" s="3"/>
@@ -21119,7 +21611,7 @@
         <f t="shared" si="4"/>
         <v>317</v>
       </c>
-      <c r="B318" s="3"/>
+      <c r="B318" s="8"/>
       <c r="C318" s="3"/>
       <c r="D318" s="3"/>
       <c r="E318" s="3"/>
@@ -21141,7 +21633,7 @@
         <f t="shared" si="4"/>
         <v>318</v>
       </c>
-      <c r="B319" s="3"/>
+      <c r="B319" s="8"/>
       <c r="C319" s="3"/>
       <c r="D319" s="3"/>
       <c r="E319" s="3"/>
@@ -21163,7 +21655,7 @@
         <f t="shared" si="4"/>
         <v>319</v>
       </c>
-      <c r="B320" s="3"/>
+      <c r="B320" s="8"/>
       <c r="C320" s="3"/>
       <c r="D320" s="3"/>
       <c r="E320" s="3"/>
@@ -21185,7 +21677,7 @@
         <f t="shared" si="4"/>
         <v>320</v>
       </c>
-      <c r="B321" s="3"/>
+      <c r="B321" s="8"/>
       <c r="C321" s="3"/>
       <c r="D321" s="3"/>
       <c r="E321" s="3"/>
@@ -21207,7 +21699,7 @@
         <f t="shared" si="4"/>
         <v>321</v>
       </c>
-      <c r="B322" s="3"/>
+      <c r="B322" s="8"/>
       <c r="C322" s="3"/>
       <c r="D322" s="3"/>
       <c r="E322" s="3"/>
@@ -21229,7 +21721,7 @@
         <f t="shared" si="4"/>
         <v>322</v>
       </c>
-      <c r="B323" s="3"/>
+      <c r="B323" s="8"/>
       <c r="C323" s="3"/>
       <c r="D323" s="3"/>
       <c r="E323" s="3"/>
@@ -21251,7 +21743,7 @@
         <f t="shared" si="4"/>
         <v>323</v>
       </c>
-      <c r="B324" s="3"/>
+      <c r="B324" s="8"/>
       <c r="C324" s="3"/>
       <c r="D324" s="3"/>
       <c r="E324" s="3"/>
@@ -21273,7 +21765,7 @@
         <f t="shared" si="4"/>
         <v>324</v>
       </c>
-      <c r="B325" s="3"/>
+      <c r="B325" s="8"/>
       <c r="C325" s="3"/>
       <c r="D325" s="3"/>
       <c r="E325" s="3"/>
@@ -21295,7 +21787,7 @@
         <f t="shared" si="4"/>
         <v>325</v>
       </c>
-      <c r="B326" s="3"/>
+      <c r="B326" s="8"/>
       <c r="C326" s="3"/>
       <c r="D326" s="3"/>
       <c r="E326" s="3"/>
@@ -21317,7 +21809,7 @@
         <f t="shared" si="4"/>
         <v>326</v>
       </c>
-      <c r="B327" s="3"/>
+      <c r="B327" s="8"/>
       <c r="C327" s="3"/>
       <c r="D327" s="3"/>
       <c r="E327" s="3"/>
@@ -21339,7 +21831,7 @@
         <f t="shared" si="4"/>
         <v>327</v>
       </c>
-      <c r="B328" s="3"/>
+      <c r="B328" s="8"/>
       <c r="C328" s="3"/>
       <c r="D328" s="3"/>
       <c r="E328" s="3"/>
@@ -21361,7 +21853,7 @@
         <f t="shared" si="4"/>
         <v>328</v>
       </c>
-      <c r="B329" s="3"/>
+      <c r="B329" s="8"/>
       <c r="C329" s="3"/>
       <c r="D329" s="3"/>
       <c r="E329" s="3"/>
@@ -21383,7 +21875,7 @@
         <f t="shared" si="4"/>
         <v>329</v>
       </c>
-      <c r="B330" s="3"/>
+      <c r="B330" s="8"/>
       <c r="C330" s="3"/>
       <c r="D330" s="3"/>
       <c r="E330" s="3"/>
@@ -21405,7 +21897,7 @@
         <f t="shared" si="4"/>
         <v>330</v>
       </c>
-      <c r="B331" s="3"/>
+      <c r="B331" s="8"/>
       <c r="C331" s="3"/>
       <c r="D331" s="3"/>
       <c r="E331" s="3"/>
@@ -21427,7 +21919,7 @@
         <f t="shared" si="4"/>
         <v>331</v>
       </c>
-      <c r="B332" s="12"/>
+      <c r="B332" s="8"/>
       <c r="C332" s="12"/>
       <c r="D332" s="12"/>
       <c r="E332" s="12"/>

</xml_diff>